<commit_message>
bug fix and new functions
</commit_message>
<xml_diff>
--- a/example_OD.xlsx
+++ b/example_OD.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\plate_reader\260323_plate3_plusNina\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipea/tools/github_famotsuka/sync-OD/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2EF103-3CD0-1748-9510-4A08C35E86A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18165" windowHeight="13170"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="18160" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -541,11 +542,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="2">
         <v>1</v>
@@ -584,7 +585,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -628,7 +629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -672,7 +673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -716,7 +717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -760,7 +761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -798,13 +799,13 @@
         <v>0.11700000000000001</v>
       </c>
       <c r="M6" s="16">
-        <v>0.11700000000000001</v>
+        <v>0.35</v>
       </c>
       <c r="N6" s="10" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -848,7 +849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -880,19 +881,19 @@
         <v>0.124</v>
       </c>
       <c r="K8" s="4">
-        <v>0.128</v>
+        <v>0.24</v>
       </c>
       <c r="L8" s="16">
         <v>0.11700000000000001</v>
       </c>
-      <c r="M8" s="16">
-        <v>0.11799999999999999</v>
+      <c r="M8" s="8">
+        <v>0.20699999999999999</v>
       </c>
       <c r="N8" s="10" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="24" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -929,8 +930,8 @@
       <c r="L9" s="15">
         <v>0.11899999999999999</v>
       </c>
-      <c r="M9" s="17">
-        <v>0.12</v>
+      <c r="M9" s="6">
+        <v>0.19500000000000001</v>
       </c>
       <c r="N9" s="10" t="s">
         <v>1</v>

</xml_diff>